<commit_message>
Update pipeline outputs, grading artifacts, and June slate data through 2026-06-09.
Refresh sport step8 outputs and caches, graded analysis reports, void validator and ticket diversity audits, mobile and ui_runner slate/ticket exports, combined ticket JSONs for late May through June, and supporting scripts for graded enrichment, stack-70 eligibility, locks/backtest tooling, and NHL/NFL data collection.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-08.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-08.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E2" t="n">
         <v>16</v>
       </c>
       <c r="F2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G2" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E6" t="n">
         <v>21</v>
       </c>
       <c r="F6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G6" t="n">
-        <v>47.7</v>
+        <v>46.7</v>
       </c>
     </row>
     <row r="7">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F7" t="n">
         <v>9</v>
       </c>
       <c r="G7" t="n">
-        <v>35.7</v>
+        <v>47.1</v>
       </c>
     </row>
     <row r="8">
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>376</v>
+        <v>402</v>
       </c>
       <c r="E8" t="n">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="F8" t="n">
-        <v>183</v>
+        <v>204</v>
       </c>
       <c r="G8" t="n">
-        <v>51.3</v>
+        <v>49.3</v>
       </c>
     </row>
     <row r="9">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>735</v>
+        <v>762</v>
       </c>
       <c r="E11" t="n">
-        <v>473</v>
+        <v>478</v>
       </c>
       <c r="F11" t="n">
-        <v>262</v>
+        <v>284</v>
       </c>
       <c r="G11" t="n">
-        <v>64.40000000000001</v>
+        <v>62.7</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E12" t="n">
         <v>142</v>
       </c>
       <c r="F12" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G12" t="n">
-        <v>67.90000000000001</v>
+        <v>67.59999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -790,16 +790,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E13" t="n">
         <v>104</v>
       </c>
       <c r="F13" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="G13" t="n">
-        <v>49.3</v>
+        <v>49.1</v>
       </c>
     </row>
     <row r="14">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="E14" t="n">
         <v>59</v>
       </c>
       <c r="F14" t="n">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="G14" t="n">
-        <v>30.6</v>
+        <v>29.5</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="E15" t="n">
         <v>57</v>
       </c>
       <c r="F15" t="n">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="G15" t="n">
-        <v>20.2</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E16" t="n">
         <v>43</v>
       </c>
       <c r="F16" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G16" t="n">
-        <v>22.2</v>
+        <v>22.1</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3072</v>
+        <v>3182</v>
       </c>
       <c r="E17" t="n">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="F17" t="n">
-        <v>2357</v>
+        <v>2463</v>
       </c>
       <c r="G17" t="n">
-        <v>23.3</v>
+        <v>22.6</v>
       </c>
     </row>
   </sheetData>
@@ -1351,10 +1351,10 @@
         <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>37.2</v>
+        <v>30.9</v>
       </c>
       <c r="Y4" t="n">
-        <v>43</v>
+        <v>68</v>
       </c>
       <c r="Z4" t="n">
         <v>66.7</v>
@@ -1564,52 +1564,52 @@
         <v>252</v>
       </c>
       <c r="D7" t="n">
-        <v>64.40000000000001</v>
+        <v>62.7</v>
       </c>
       <c r="E7" t="n">
-        <v>735</v>
+        <v>762</v>
       </c>
       <c r="F7" t="n">
-        <v>67.90000000000001</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="H7" t="n">
-        <v>49.3</v>
+        <v>49.1</v>
       </c>
       <c r="I7" t="n">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J7" t="n">
-        <v>30.6</v>
+        <v>29.5</v>
       </c>
       <c r="K7" t="n">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="L7" t="n">
-        <v>20.2</v>
+        <v>19.9</v>
       </c>
       <c r="M7" t="n">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="N7" t="n">
-        <v>22.2</v>
+        <v>22.1</v>
       </c>
       <c r="O7" t="n">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="P7" t="n">
-        <v>23.3</v>
+        <v>22.6</v>
       </c>
       <c r="Q7" t="n">
-        <v>3072</v>
+        <v>3182</v>
       </c>
       <c r="R7" t="n">
+        <v>39</v>
+      </c>
+      <c r="S7" t="n">
         <v>41</v>
-      </c>
-      <c r="S7" t="n">
-        <v>39</v>
       </c>
       <c r="T7" t="n">
         <v>47.1</v>
@@ -1618,16 +1618,16 @@
         <v>34</v>
       </c>
       <c r="V7" t="n">
-        <v>47.7</v>
+        <v>46.7</v>
       </c>
       <c r="W7" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="X7" t="n">
-        <v>51.3</v>
+        <v>49.3</v>
       </c>
       <c r="Y7" t="n">
-        <v>376</v>
+        <v>402</v>
       </c>
       <c r="Z7" t="n">
         <v>49.6</v>
@@ -1642,10 +1642,10 @@
         <v>80</v>
       </c>
       <c r="AD7" t="n">
-        <v>35.7</v>
+        <v>47.1</v>
       </c>
       <c r="AE7" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="AF7" t="n">
         <v>53.7</v>

</xml_diff>